<commit_message>
a lot of update on the site
</commit_message>
<xml_diff>
--- a/files/unmapped_drg_price.xlsx
+++ b/files/unmapped_drg_price.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aquacy\Documents\last\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0B96EBA-40BB-416F-ACF4-AF9816BDBDA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E66F1762-40AD-448A-AEDB-3D13982CF3A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4845" yWindow="1800" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -1062,6 +1062,7 @@
   <dimension ref="A1:AA111"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="3" width="51.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.5703125" customWidth="1"/>

</xml_diff>